<commit_message>
Add HSR 4.6 confirmed banner
</commit_message>
<xml_diff>
--- a/banners/03_Honkai_Star_Rail_confirmed.xlsx
+++ b/banners/03_Honkai_Star_Rail_confirmed.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -459,6 +459,33 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>4.6 Phase 1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>2026-10-21</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>3.89,3.26</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3.84,3.61,3.54</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>